<commit_message>
Added email notifications and late punch WhatsApp report
</commit_message>
<xml_diff>
--- a/uploads/Sample_Attendance.xlsx
+++ b/uploads/Sample_Attendance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maharajan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D6A39ED-56CA-4C9E-A3B0-2ACE49F03979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F75823B-73EF-4F61-B9F6-91324EE5803D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5604" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>Employee ID</t>
   </si>
@@ -65,9 +65,6 @@
     <t>15-07-2026</t>
   </si>
   <si>
-    <t>08:55</t>
-  </si>
-  <si>
     <t>17:50</t>
   </si>
   <si>
@@ -80,9 +77,6 @@
     <t>9600788865</t>
   </si>
   <si>
-    <t>09:10</t>
-  </si>
-  <si>
     <t>18:30</t>
   </si>
   <si>
@@ -96,16 +90,33 @@
   </si>
   <si>
     <t>Vikram</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>maharajan4m2p@gmail.com</t>
+  </si>
+  <si>
+    <t>maharajan0731@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -128,14 +139,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -436,14 +451,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.77734375" customWidth="1"/>
+    <col min="7" max="7" width="24.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -462,8 +479,11 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -476,39 +496,45 @@
       <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3">
+        <v>0.41319444444444442</v>
+      </c>
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
       </c>
       <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3">
+        <v>0.3923611111111111</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
       </c>
       <c r="C4">
         <v>8870363966</v>
@@ -520,12 +546,12 @@
         <v>8.5500000000000007</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C5">
         <v>9585328220</v>
@@ -541,6 +567,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{B018042C-18EC-4E33-85FE-456D1687AD59}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{9BC7A5CF-27AB-4258-8D1F-945D28C3563E}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
LATE PUNCING AND MISSING REPORT
</commit_message>
<xml_diff>
--- a/uploads/Sample_Attendance.xlsx
+++ b/uploads/Sample_Attendance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maharajan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F75823B-73EF-4F61-B9F6-91324EE5803D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEEC7B11-7F3C-4251-8794-EB191B959FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5604" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>Employee ID</t>
   </si>
@@ -99,6 +99,21 @@
   </si>
   <si>
     <t>maharajan0731@gmail.com</t>
+  </si>
+  <si>
+    <t>EMPOO6</t>
+  </si>
+  <si>
+    <t>Maharajan</t>
+  </si>
+  <si>
+    <t>msjhdvsnkxkdjj@gmail.com</t>
+  </si>
+  <si>
+    <t>EMP009</t>
+  </si>
+  <si>
+    <t>VIRAT</t>
   </si>
 </sst>
 </file>
@@ -451,7 +466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="11.44140625" bestFit="1" customWidth="1"/>
@@ -566,10 +581,51 @@
         <v>4.3</v>
       </c>
     </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>9512984169</v>
+      </c>
+      <c r="D6" s="1">
+        <v>46218</v>
+      </c>
+      <c r="E6">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7">
+        <v>4826950827</v>
+      </c>
+      <c r="D7" s="1">
+        <v>46218</v>
+      </c>
+      <c r="E7">
+        <v>9.5500000000000007</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" xr:uid="{B018042C-18EC-4E33-85FE-456D1687AD59}"/>
     <hyperlink ref="G3" r:id="rId2" xr:uid="{9BC7A5CF-27AB-4258-8D1F-945D28C3563E}"/>
+    <hyperlink ref="G6" r:id="rId3" xr:uid="{0FD0E123-4368-448D-B018-FADB0F6AC8A1}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>